<commit_message>
A data do corte passa a ser justificada pela guerra, não pelo PPI
Ele escolheu março porque foi quando a guerra começou. É justificativa melhor
que a minha: a guerra é exógena ao preço brasileiro, enquanto o salto do PPI
já é a transmissão dela, e justificar o corte pelo próprio dado chega perto de
escolher a data pelo resultado.

A série passa a confirmar a data em vez de escolhê-la, e confirma bem: o PPI
de Paulínia atravessa fevereiro inteiro parado entre R$ 2,46 e R$ 2,60, e faz
+15,7% na semana encerrada em 6/3, +16,4% na seguinte e +13,2% na outra,
chegando a R$ 4,04 em 27/3. São 55% em quatro semanas, com a tabela da
Petrobras em R$ 2,5808 o tempo todo.

Isso também resolve o "talvez final de fevereiro": para o preço não dá no
mesmo, dá em nada. Fevereiro não tem movimento de PPI nenhum. Qualquer que
tenha sido o dia da guerra, a transmissão para a paridade brasileira começa na
primeira semana de março.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/ipca-defasagem.xlsx
+++ b/planilhas/ipca-defasagem.xlsx
@@ -15214,7 +15214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15285,45 +15285,45 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>de fora são justamente os de contribuição negativa, e o número sobe sozinho. Por isso março de 2026 não</t>
+          <t>de fora são justamente os de contribuição negativa, e o número sobe sozinho.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>foi escolhido pelo gráfico: é o mês em que o PPI salta. Em Paulínia ele sai de R$ 2,573 em fevereiro para</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>R$ 3,630 em março, enquanto a tabela da Petrobras fica em R$ 2,5808, onde estava desde 27/1/2026 e onde</t>
+          <t>Por isso o corte vem de fora dos dados: março de 2026 é quando começa a guerra no Oriente Médio. A série</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ficaria até maio. O choque está no PPI, e a data vem dele.</t>
+          <t>confirma a data em vez de escolhê-la. O PPI de Paulínia passa fevereiro inteiro parado entre R$ 2,46 e</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>R$ 2,60, e aí faz +15,7% na semana encerrada em 6/3, +16,4% na seguinte e +13,2% na outra, chegando a</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>E a tabela de baixo varre o corte mês a mês, para você ver quanto a escolha decide. Ela anda MUITO:</t>
+          <t>R$ 4,04 em 27/3: 55% em quatro semanas. A tabela da Petrobras fica em R$ 2,5808 o tempo todo, onde</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cortando em março o contábil dá +0,70 p.p., cortando em abril dá +0,08. Quase todo o efeito está num mês só.</t>
+          <t>estava desde 27/1/2026 e onde ficaria até maio.</t>
         </is>
       </c>
     </row>
@@ -15333,194 +15333,127 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Isso não é defeito da conta, é o que a conta mede. O efeito no acumulado em doze meses é a MUDANÇA do</t>
+          <t>E a tabela de baixo varre o corte mês a mês, para você ver quanto a escolha decide. Ela anda MUITO:</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>represamento, não o nível dele. Março é o mês em que a defasagem abre; quem começa a contar em abril já</t>
+          <t>cortando em março o contábil dá +0,70 p.p., cortando em abril dá +0,08. Quase todo o efeito está num mês só.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>encontra a defasagem aberta nas duas pontas da comparação, e por isso não vê nada.</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Isso não é defeito da conta, é o que a conta mede. O efeito no acumulado em doze meses é a MUDANÇA do</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>A consequência para quem for citar o número: ele é 'o efeito de a defasagem TER ABERTO em março', não</t>
+          <t>represamento, não o nível dele. Março é o mês em que a defasagem abre; quem começa a contar em abril já</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>encontra a defasagem aberta nas duas pontas da comparação, e por isso não vê nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>A consequência para quem for citar o número: ele é 'o efeito de a defasagem TER ABERTO em março', não</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>'o efeito de a defasagem existir'. Para o segundo, a coluna certa é 'nível represado' da aba Modelo</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>mensal, que em setembro de 2026 está em 0,63 p.p. e não depende de data de corte nenhuma.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>mês</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>IPCA 12m observado %</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>contrafactual contábil %</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>contrafactual Bahia %</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>contrafactual Salvador %</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>efeito contábil (p.p.)</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>efeito Bahia (p.p.)</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>efeito Salvador (p.p.)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2021-12</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="n">
-        <v>10.0610548932579</v>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>10.0610548932579</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>10.0610548932579</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>10.0610548932579</v>
-      </c>
-      <c r="F27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="3" t="n">
-        <v>0</v>
+          <t>mensal, que em setembro de 2026 está em 0,63 p.p. e não depende de data de corte nenhuma.</t>
+        </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2022-01</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="n">
-        <v>10.3794359996823</v>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>10.3794359996823</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>10.3794359996823</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>10.3794359996823</v>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2022-02</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n">
-        <v>10.54359340003879</v>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>10.54359340003879</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>10.54359340003879</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>10.54359340003879</v>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="3" t="n">
-        <v>0</v>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>mês</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>IPCA 12m observado %</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>contrafactual contábil %</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>contrafactual Bahia %</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>contrafactual Salvador %</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>efeito contábil (p.p.)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>efeito Bahia (p.p.)</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>efeito Salvador (p.p.)</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2022-03</t>
+          <t>2021-12</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>11.299315974556</v>
+        <v>10.0610548932579</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>11.299315974556</v>
+        <v>10.0610548932579</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>11.299315974556</v>
+        <v>10.0610548932579</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>11.299315974556</v>
+        <v>10.0610548932579</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>0</v>
@@ -15535,20 +15468,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2022-04</t>
+          <t>2022-01</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>12.13148113237592</v>
+        <v>10.3794359996823</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>12.13148113237592</v>
+        <v>10.3794359996823</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>12.13148113237592</v>
+        <v>10.3794359996823</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>12.13148113237592</v>
+        <v>10.3794359996823</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0</v>
@@ -15563,20 +15496,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2022-05</t>
+          <t>2022-02</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>11.73113070881493</v>
+        <v>10.54359340003879</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>11.73113070881493</v>
+        <v>10.54359340003879</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>11.73113070881493</v>
+        <v>10.54359340003879</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>11.73113070881493</v>
+        <v>10.54359340003879</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0</v>
@@ -15591,20 +15524,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2022-06</t>
+          <t>2022-03</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>11.88672961759074</v>
+        <v>11.299315974556</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>11.88672961759074</v>
+        <v>11.299315974556</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>11.88672961759074</v>
+        <v>11.299315974556</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>11.88672961759074</v>
+        <v>11.299315974556</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0</v>
@@ -15619,20 +15552,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2022-07</t>
+          <t>2022-04</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>10.06923519828753</v>
+        <v>12.13148113237592</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>10.06923519828753</v>
+        <v>12.13148113237592</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>10.06923519828753</v>
+        <v>12.13148113237592</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>10.06923519828753</v>
+        <v>12.13148113237592</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>0</v>
@@ -15647,20 +15580,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2022-08</t>
+          <t>2022-05</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>8.727060525006136</v>
+        <v>11.73113070881493</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>8.727060525006136</v>
+        <v>11.73113070881493</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>8.727060525006136</v>
+        <v>11.73113070881493</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>8.727060525006136</v>
+        <v>11.73113070881493</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0</v>
@@ -15675,20 +15608,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2022-09</t>
+          <t>2022-06</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>7.168596332032062</v>
+        <v>11.88672961759074</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>7.168596332032062</v>
+        <v>11.88672961759074</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>7.168596332032062</v>
+        <v>11.88672961759074</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>7.168596332032062</v>
+        <v>11.88672961759074</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0</v>
@@ -15703,20 +15636,20 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2022-10</t>
+          <t>2022-07</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>6.470015852238076</v>
+        <v>10.06923519828753</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>6.470015852238076</v>
+        <v>10.06923519828753</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>6.470015852238076</v>
+        <v>10.06923519828753</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>6.470015852238076</v>
+        <v>10.06923519828753</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>0</v>
@@ -15731,20 +15664,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2022-11</t>
+          <t>2022-08</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>5.900488278585692</v>
+        <v>8.727060525006136</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>5.900488278585692</v>
+        <v>8.727060525006136</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>5.900488278585692</v>
+        <v>8.727060525006136</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>5.900488278585692</v>
+        <v>8.727060525006136</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>0</v>
@@ -15759,20 +15692,20 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2022-12</t>
+          <t>2022-09</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>5.784841959607756</v>
+        <v>7.168596332032062</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>5.784841959607756</v>
+        <v>7.168596332032062</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>5.784841959607756</v>
+        <v>7.168596332032062</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>5.784841959607756</v>
+        <v>7.168596332032062</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0</v>
@@ -15787,20 +15720,20 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2022-10</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>5.774320292414625</v>
+        <v>6.470015852238076</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>5.774320292414625</v>
+        <v>6.470015852238076</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>5.774320292414625</v>
+        <v>6.470015852238076</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>5.774320292414625</v>
+        <v>6.470015852238076</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>0</v>
@@ -15815,20 +15748,20 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2023-02</t>
+          <t>2022-11</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>5.596301933344128</v>
+        <v>5.900488278585692</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>5.596301933344128</v>
+        <v>5.900488278585692</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>5.596301933344128</v>
+        <v>5.900488278585692</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>5.596301933344128</v>
+        <v>5.900488278585692</v>
       </c>
       <c r="F41" s="3" t="n">
         <v>0</v>
@@ -15843,20 +15776,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2023-03</t>
+          <t>2022-12</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>4.65069442734789</v>
+        <v>5.784841959607756</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>4.65069442734789</v>
+        <v>5.784841959607756</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>4.65069442734789</v>
+        <v>5.784841959607756</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>4.65069442734789</v>
+        <v>5.784841959607756</v>
       </c>
       <c r="F42" s="3" t="n">
         <v>0</v>
@@ -15871,20 +15804,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2023-04</t>
+          <t>2023-01</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>4.184705782064824</v>
+        <v>5.774320292414625</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>4.184705782064824</v>
+        <v>5.774320292414625</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>4.184705782064824</v>
+        <v>5.774320292414625</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>4.184705782064824</v>
+        <v>5.774320292414625</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>0</v>
@@ -15899,20 +15832,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2023-05</t>
+          <t>2023-02</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>3.935832194051536</v>
+        <v>5.596301933344128</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>3.935832194051536</v>
+        <v>5.596301933344128</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>3.935832194051536</v>
+        <v>5.596301933344128</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>3.935832194051536</v>
+        <v>5.596301933344128</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0</v>
@@ -15927,20 +15860,20 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2023-06</t>
+          <t>2023-03</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>3.161501468457617</v>
+        <v>4.65069442734789</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>3.161501468457617</v>
+        <v>4.65069442734789</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>3.161501468457617</v>
+        <v>4.65069442734789</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>3.161501468457617</v>
+        <v>4.65069442734789</v>
       </c>
       <c r="F45" s="3" t="n">
         <v>0</v>
@@ -15955,20 +15888,20 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2023-07</t>
+          <t>2023-04</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>3.992443888662711</v>
+        <v>4.184705782064824</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>3.992443888662711</v>
+        <v>4.184705782064824</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>3.992443888662711</v>
+        <v>4.184705782064824</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>3.992443888662711</v>
+        <v>4.184705782064824</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>0</v>
@@ -15983,20 +15916,20 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2023-05</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>4.608216087521688</v>
+        <v>3.935832194051536</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>4.608216087521688</v>
+        <v>3.935832194051536</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>4.608216087521688</v>
+        <v>3.935832194051536</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>4.608216087521688</v>
+        <v>3.935832194051536</v>
       </c>
       <c r="F47" s="3" t="n">
         <v>0</v>
@@ -16011,20 +15944,20 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2023-06</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>5.185234629775626</v>
+        <v>3.161501468457617</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>5.185234629775626</v>
+        <v>3.161501468457617</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>5.185234629775626</v>
+        <v>3.161501468457617</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>5.185234629775626</v>
+        <v>3.161501468457617</v>
       </c>
       <c r="F48" s="3" t="n">
         <v>0</v>
@@ -16039,20 +15972,20 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2023-07</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>4.819245643589931</v>
+        <v>3.992443888662711</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>4.819245643589931</v>
+        <v>3.992443888662711</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>4.819245643589931</v>
+        <v>3.992443888662711</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>4.819245643589931</v>
+        <v>3.992443888662711</v>
       </c>
       <c r="F49" s="3" t="n">
         <v>0</v>
@@ -16067,20 +16000,20 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-08</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>4.683537029570672</v>
+        <v>4.608216087521688</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>4.683537029570672</v>
+        <v>4.608216087521688</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>4.683537029570672</v>
+        <v>4.608216087521688</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>4.683537029570672</v>
+        <v>4.608216087521688</v>
       </c>
       <c r="F50" s="3" t="n">
         <v>0</v>
@@ -16095,20 +16028,20 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>4.621113930566789</v>
+        <v>5.185234629775626</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>4.621113930566789</v>
+        <v>5.185234629775626</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>4.621113930566789</v>
+        <v>5.185234629775626</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>4.621113930566789</v>
+        <v>5.185234629775626</v>
       </c>
       <c r="F51" s="3" t="n">
         <v>0</v>
@@ -16123,20 +16056,20 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>4.506637430692439</v>
+        <v>4.819245643589931</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>4.506637430692439</v>
+        <v>4.819245643589931</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>4.506637430692439</v>
+        <v>4.819245643589931</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>4.506637430692439</v>
+        <v>4.819245643589931</v>
       </c>
       <c r="F52" s="3" t="n">
         <v>0</v>
@@ -16151,20 +16084,20 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>4.496273821268559</v>
+        <v>4.683537029570672</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>4.496273821268559</v>
+        <v>4.683537029570672</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>4.496273821268559</v>
+        <v>4.683537029570672</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>4.496273821268559</v>
+        <v>4.683537029570672</v>
       </c>
       <c r="F53" s="3" t="n">
         <v>0</v>
@@ -16179,20 +16112,20 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>3.925596126881703</v>
+        <v>4.621113930566789</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>3.925596126881703</v>
+        <v>4.621113930566789</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>3.925596126881703</v>
+        <v>4.621113930566789</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>3.925596126881703</v>
+        <v>4.621113930566789</v>
       </c>
       <c r="F54" s="3" t="n">
         <v>0</v>
@@ -16207,20 +16140,20 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>3.688016491565316</v>
+        <v>4.506637430692439</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>3.688016491565316</v>
+        <v>4.506637430692439</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>3.688016491565316</v>
+        <v>4.506637430692439</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>3.688016491565316</v>
+        <v>4.506637430692439</v>
       </c>
       <c r="F55" s="3" t="n">
         <v>0</v>
@@ -16235,20 +16168,20 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>3.92595167856582</v>
+        <v>4.496273821268559</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>3.92595167856582</v>
+        <v>4.496273821268559</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>3.92595167856582</v>
+        <v>4.496273821268559</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>3.92595167856582</v>
+        <v>4.496273821268559</v>
       </c>
       <c r="F56" s="3" t="n">
         <v>0</v>
@@ -16263,20 +16196,20 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>4.227578239682583</v>
+        <v>3.925596126881703</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>4.227578239682583</v>
+        <v>3.925596126881703</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>4.227578239682583</v>
+        <v>3.925596126881703</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>4.227578239682583</v>
+        <v>3.925596126881703</v>
       </c>
       <c r="F57" s="3" t="n">
         <v>0</v>
@@ -16291,20 +16224,20 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>4.498245142821999</v>
+        <v>3.688016491565316</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>4.498245142821999</v>
+        <v>3.688016491565316</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>4.498245142821999</v>
+        <v>3.688016491565316</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>4.498245142821999</v>
+        <v>3.688016491565316</v>
       </c>
       <c r="F58" s="3" t="n">
         <v>0</v>
@@ -16319,20 +16252,20 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>4.237599016056492</v>
+        <v>3.92595167856582</v>
       </c>
       <c r="C59" s="3" t="n">
-        <v>4.237599016056492</v>
+        <v>3.92595167856582</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>4.237599016056492</v>
+        <v>3.92595167856582</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>4.237599016056492</v>
+        <v>3.92595167856582</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>0</v>
@@ -16347,20 +16280,20 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
-        <v>4.424740127395888</v>
+        <v>4.227578239682583</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>4.424740127395888</v>
+        <v>4.227578239682583</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>4.424740127395888</v>
+        <v>4.227578239682583</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>4.424740127395888</v>
+        <v>4.227578239682583</v>
       </c>
       <c r="F60" s="3" t="n">
         <v>0</v>
@@ -16375,20 +16308,20 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>4.758099233947855</v>
+        <v>4.498245142821999</v>
       </c>
       <c r="C61" s="3" t="n">
-        <v>4.758099233947855</v>
+        <v>4.498245142821999</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>4.758099233947855</v>
+        <v>4.498245142821999</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>4.758099233947855</v>
+        <v>4.498245142821999</v>
       </c>
       <c r="F61" s="3" t="n">
         <v>0</v>
@@ -16403,20 +16336,20 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B62" s="3" t="n">
-        <v>4.87301138907088</v>
+        <v>4.237599016056492</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>4.87301138907088</v>
+        <v>4.237599016056492</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>4.87301138907088</v>
+        <v>4.237599016056492</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>4.87301138907088</v>
+        <v>4.237599016056492</v>
       </c>
       <c r="F62" s="3" t="n">
         <v>0</v>
@@ -16431,20 +16364,20 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>4.831295791859591</v>
+        <v>4.424740127395888</v>
       </c>
       <c r="C63" s="3" t="n">
-        <v>4.831295791859591</v>
+        <v>4.424740127395888</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>4.831295791859591</v>
+        <v>4.424740127395888</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>4.831295791859591</v>
+        <v>4.424740127395888</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>0</v>
@@ -16459,20 +16392,20 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
-        <v>4.559874392677332</v>
+        <v>4.758099233947855</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>4.559874392677332</v>
+        <v>4.758099233947855</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>4.559874392677332</v>
+        <v>4.758099233947855</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>4.559874392677332</v>
+        <v>4.758099233947855</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>0</v>
@@ -16487,20 +16420,20 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
-        <v>5.057630414778758</v>
+        <v>4.87301138907088</v>
       </c>
       <c r="C65" s="3" t="n">
-        <v>5.057630414778758</v>
+        <v>4.87301138907088</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>5.057630414778758</v>
+        <v>4.87301138907088</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>5.057630414778758</v>
+        <v>4.87301138907088</v>
       </c>
       <c r="F65" s="3" t="n">
         <v>0</v>
@@ -16515,20 +16448,20 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B66" s="3" t="n">
-        <v>5.477189641674851</v>
+        <v>4.831295791859591</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>5.477189641674851</v>
+        <v>4.831295791859591</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>5.477189641674851</v>
+        <v>4.831295791859591</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>5.477189641674851</v>
+        <v>4.831295791859591</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>0</v>
@@ -16543,20 +16476,20 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B67" s="3" t="n">
-        <v>5.52972858849774</v>
+        <v>4.559874392677332</v>
       </c>
       <c r="C67" s="3" t="n">
-        <v>5.52972858849774</v>
+        <v>4.559874392677332</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>5.52972858849774</v>
+        <v>4.559874392677332</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>5.52972858849774</v>
+        <v>4.559874392677332</v>
       </c>
       <c r="F67" s="3" t="n">
         <v>0</v>
@@ -16571,20 +16504,20 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B68" s="3" t="n">
-        <v>5.319635559255276</v>
+        <v>5.057630414778758</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>5.319635559255276</v>
+        <v>5.057630414778758</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>5.319635559255276</v>
+        <v>5.057630414778758</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>5.319635559255276</v>
+        <v>5.057630414778758</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>0</v>
@@ -16599,20 +16532,20 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>5.35116523759851</v>
+        <v>5.477189641674851</v>
       </c>
       <c r="C69" s="3" t="n">
-        <v>5.35116523759851</v>
+        <v>5.477189641674851</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>5.35116523759851</v>
+        <v>5.477189641674851</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>5.35116523759851</v>
+        <v>5.477189641674851</v>
       </c>
       <c r="F69" s="3" t="n">
         <v>0</v>
@@ -16627,20 +16560,20 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B70" s="3" t="n">
-        <v>5.225222422012621</v>
+        <v>5.52972858849774</v>
       </c>
       <c r="C70" s="3" t="n">
-        <v>5.225222422012621</v>
+        <v>5.52972858849774</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>5.225222422012621</v>
+        <v>5.52972858849774</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>5.225222422012621</v>
+        <v>5.52972858849774</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>0</v>
@@ -16655,20 +16588,20 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B71" s="3" t="n">
-        <v>5.130500777503921</v>
+        <v>5.319635559255276</v>
       </c>
       <c r="C71" s="3" t="n">
-        <v>5.130500777503921</v>
+        <v>5.319635559255276</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>5.130500777503921</v>
+        <v>5.319635559255276</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>5.130500777503921</v>
+        <v>5.319635559255276</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>0</v>
@@ -16683,20 +16616,20 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B72" s="3" t="n">
-        <v>5.172368758697643</v>
+        <v>5.35116523759851</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>5.172368758697643</v>
+        <v>5.35116523759851</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>5.172368758697643</v>
+        <v>5.35116523759851</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>5.172368758697643</v>
+        <v>5.35116523759851</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>0</v>
@@ -16711,20 +16644,20 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>4.680811347037062</v>
+        <v>5.225222422012621</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>4.680811347037062</v>
+        <v>5.225222422012621</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>4.680811347037062</v>
+        <v>5.225222422012621</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>4.680811347037062</v>
+        <v>5.225222422012621</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>0</v>
@@ -16739,20 +16672,20 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="B74" s="3" t="n">
-        <v>4.461835648432833</v>
+        <v>5.130500777503921</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>4.461835648432833</v>
+        <v>5.130500777503921</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>4.461835648432833</v>
+        <v>5.130500777503921</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>4.461835648432833</v>
+        <v>5.130500777503921</v>
       </c>
       <c r="F74" s="3" t="n">
         <v>0</v>
@@ -16767,20 +16700,20 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>4.264384904568952</v>
+        <v>5.172368758697643</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>4.264384904568952</v>
+        <v>5.172368758697643</v>
       </c>
       <c r="D75" s="3" t="n">
-        <v>4.264384904568952</v>
+        <v>5.172368758697643</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>4.264384904568952</v>
+        <v>5.172368758697643</v>
       </c>
       <c r="F75" s="3" t="n">
         <v>0</v>
@@ -16795,20 +16728,20 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="B76" s="3" t="n">
-        <v>4.44135121281346</v>
+        <v>4.680811347037062</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>4.44135121281346</v>
+        <v>4.680811347037062</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>4.44135121281346</v>
+        <v>4.680811347037062</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>4.44135121281346</v>
+        <v>4.680811347037062</v>
       </c>
       <c r="F76" s="3" t="n">
         <v>0</v>
@@ -16823,20 +16756,20 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B77" s="3" t="n">
-        <v>3.812496961112588</v>
+        <v>4.461835648432833</v>
       </c>
       <c r="C77" s="3" t="n">
-        <v>3.812496961112588</v>
+        <v>4.461835648432833</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>3.812496961112588</v>
+        <v>4.461835648432833</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>3.812496961112588</v>
+        <v>4.461835648432833</v>
       </c>
       <c r="F77" s="3" t="n">
         <v>0</v>
@@ -16851,307 +16784,328 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="B78" s="3" t="n">
-        <v>4.142846991219562</v>
+        <v>4.264384904568952</v>
       </c>
       <c r="C78" s="3" t="n">
-        <v>4.759406247070297</v>
+        <v>4.264384904568952</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>4.373166150937546</v>
+        <v>4.264384904568952</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>4.792271706483553</v>
+        <v>4.264384904568952</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>0.6165592558507349</v>
+        <v>0</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>0.2303191597179843</v>
+        <v>0</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>0.6494247152639909</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B79" s="3" t="n">
-        <v>4.39171967147336</v>
+        <v>4.44135121281346</v>
       </c>
       <c r="C79" s="3" t="n">
-        <v>5.249294436370278</v>
+        <v>4.44135121281346</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>4.71778514034904</v>
+        <v>4.44135121281346</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>4.980916293512805</v>
+        <v>4.44135121281346</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>0.8575747648969179</v>
+        <v>0</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>0.3260654688756803</v>
+        <v>0</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>0.5891966220394451</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B80" s="3" t="n">
-        <v>4.724906887660008</v>
+        <v>3.812496961112588</v>
       </c>
       <c r="C80" s="3" t="n">
-        <v>5.611456542936688</v>
+        <v>3.812496961112588</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>5.062685247756948</v>
+        <v>3.812496961112588</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>5.205248811719421</v>
+        <v>3.812496961112588</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>0.8865496552766805</v>
+        <v>0</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>0.3377783600969408</v>
+        <v>0</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>0.4803419240594131</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B81" s="3" t="n">
-        <v>4.641327552554153</v>
+        <v>4.142846991219562</v>
       </c>
       <c r="C81" s="3" t="n">
-        <v>5.108953246822145</v>
+        <v>4.759406247070297</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>4.80827557603456</v>
+        <v>4.373166150937546</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>5.236553842569913</v>
+        <v>4.792271706483553</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>0.4676256942679924</v>
+        <v>0.6165592558507349</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>0.1669480234804066</v>
+        <v>0.2303191597179843</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>0.5952262900157601</v>
+        <v>0.6494247152639909</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B82" s="3" t="n">
-        <v>4.44302461783459</v>
+        <v>4.39171967147336</v>
       </c>
       <c r="C82" s="3" t="n">
-        <v>5.024469608744919</v>
+        <v>5.249294436370278</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>4.654371701684279</v>
+        <v>4.71778514034904</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>4.923999691256942</v>
+        <v>4.980916293512805</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>0.5814449909103292</v>
+        <v>0.8575747648969179</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>0.2113470838496889</v>
+        <v>0.3260654688756803</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>0.4809750734223517</v>
+        <v>0.5891966220394451</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B83" s="3" t="n">
-        <v>4.223452737068278</v>
+        <v>4.724906887660008</v>
       </c>
       <c r="C83" s="3" t="n">
-        <v>4.780929656596666</v>
+        <v>5.611456542936688</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>4.430692099619438</v>
+        <v>5.062685247756948</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>4.500631240168573</v>
+        <v>5.205248811719421</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>0.557476919528388</v>
+        <v>0.8865496552766805</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>0.2072393625511593</v>
+        <v>0.3377783600969408</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>0.2771785031002949</v>
+        <v>0.4803419240594131</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>4.641327552554153</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>5.108953246822145</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>4.80827557603456</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>5.236553842569913</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0.4676256942679924</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0.1669480234804066</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0.5952262900157601</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>4.44302461783459</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>5.024469608744919</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>4.654371701684279</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>4.923999691256942</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0.5814449909103292</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>0.2113470838496889</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>0.4809750734223517</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>4.223452737068278</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>4.780929656596666</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>4.430692099619438</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>4.500631240168573</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0.557476919528388</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0.2072393625511593</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0.2771785031002949</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="B84" s="3" t="n">
+      <c r="B87" s="3" t="n">
         <v>4.576119675071877</v>
       </c>
-      <c r="C84" s="3" t="n">
+      <c r="C87" s="3" t="n">
         <v>5.27333430542396</v>
       </c>
-      <c r="D84" s="3" t="n">
+      <c r="D87" s="3" t="n">
         <v>4.839858211590276</v>
       </c>
-      <c r="E84" s="3" t="n">
+      <c r="E87" s="3" t="n">
         <v>4.771653553462518</v>
       </c>
-      <c r="F84" s="3" t="n">
+      <c r="F87" s="3" t="n">
         <v>0.6972146303520832</v>
       </c>
-      <c r="G84" s="3" t="n">
+      <c r="G87" s="3" t="n">
         <v>0.2637385365183986</v>
       </c>
-      <c r="H84" s="3" t="n">
+      <c r="H87" s="3" t="n">
         <v>0.1955338783906413</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="1" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="1" t="inlineStr">
         <is>
           <t>Sensibilidade à data de corte</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>O mesmo efeito, no último mês disponível, mudando só o mês em que o contrafactual começa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>corte</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>até</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>efeito contábil (p.p.)</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>efeito Bahia (p.p.)</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>efeito Salvador (p.p.)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="C91" s="3" t="n">
-        <v>0.7998821623593111</v>
-      </c>
-      <c r="D91" s="3" t="n">
-        <v>0.3008129217675348</v>
-      </c>
-      <c r="E91" s="3" t="n">
-        <v>-0.003640950315886293</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="C92" s="3" t="n">
-        <v>0.8346004372976612</v>
-      </c>
-      <c r="D92" s="3" t="n">
-        <v>0.313570975286348</v>
-      </c>
-      <c r="E92" s="3" t="n">
-        <v>-0.06206449954266891</v>
+          <t>O mesmo efeito, no último mês disponível, mudando só o mês em que o contrafactual começa.</t>
+        </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="n">
-        <v>0.7689093217567278</v>
-      </c>
-      <c r="D93" s="3" t="n">
-        <v>0.2895200110215157</v>
-      </c>
-      <c r="E93" s="3" t="n">
-        <v>0.0422933750593435</v>
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>corte</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>até</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>efeito contábil (p.p.)</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>efeito Bahia (p.p.)</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>efeito Salvador (p.p.)</t>
+        </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -17160,19 +17114,19 @@
         </is>
       </c>
       <c r="C94" s="3" t="n">
-        <v>0.8645159525793034</v>
+        <v>0.7998821623593111</v>
       </c>
       <c r="D94" s="3" t="n">
-        <v>0.3247744007882414</v>
+        <v>0.3008129217675348</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>0.1039358582213268</v>
+        <v>-0.003640950315886293</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -17181,19 +17135,19 @@
         </is>
       </c>
       <c r="C95" s="3" t="n">
-        <v>0.8670809847609817</v>
+        <v>0.8346004372976612</v>
       </c>
       <c r="D95" s="3" t="n">
-        <v>0.325709506093963</v>
+        <v>0.313570975286348</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>0.03689135095714668</v>
+        <v>-0.06206449954266891</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -17202,19 +17156,19 @@
         </is>
       </c>
       <c r="C96" s="3" t="n">
-        <v>0.6972146303520832</v>
+        <v>0.7689093217567278</v>
       </c>
       <c r="D96" s="3" t="n">
-        <v>0.2637385365183986</v>
+        <v>0.2895200110215157</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>0.1955338783906413</v>
+        <v>0.0422933750593435</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -17223,19 +17177,19 @@
         </is>
       </c>
       <c r="C97" s="3" t="n">
-        <v>0.07763066185193512</v>
+        <v>0.8645159525793034</v>
       </c>
       <c r="D97" s="3" t="n">
-        <v>0.03238953237565401</v>
+        <v>0.3247744007882414</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>-0.4537630608652865</v>
+        <v>0.1039358582213268</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -17244,33 +17198,96 @@
         </is>
       </c>
       <c r="C98" s="3" t="n">
-        <v>-0.1605560122005079</v>
+        <v>0.8670809847609817</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>-0.06270703792539134</v>
+        <v>0.325709506093963</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>-0.3924882740031777</v>
+        <v>0.03689135095714668</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="n">
+        <v>0.6972146303520832</v>
+      </c>
+      <c r="D99" s="3" t="n">
+        <v>0.2637385365183986</v>
+      </c>
+      <c r="E99" s="3" t="n">
+        <v>0.1955338783906413</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>0.07763066185193512</v>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>0.03238953237565401</v>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>-0.4537630608652865</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="n">
+        <v>-0.1605560122005079</v>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>-0.06270703792539134</v>
+      </c>
+      <c r="E101" s="3" t="n">
+        <v>-0.3924882740031777</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="C99" s="3" t="n">
+      <c r="C102" s="3" t="n">
         <v>-0.1864966761041753</v>
       </c>
-      <c r="D99" s="3" t="n">
+      <c r="D102" s="3" t="n">
         <v>-0.07332343078234604</v>
       </c>
-      <c r="E99" s="3" t="n">
+      <c r="E102" s="3" t="n">
         <v>-0.2828283537525733</v>
       </c>
     </row>

</xml_diff>